<commit_message>
PBStools 1.45.0 (2026-04-10)  [Rcheck=T, Rbuild=T]   * R code     + Added new function `collateGBSP' to collate results from `fos_gfb_offloads.sql' (RH 260227)       - creates tables of species samples by fishing year and port and dumps them to CSV files     + Changed LRP from 0.16B0 to 0.2B0 for SGR 2025 (RH 260312)     + Tweaked function `splineCPUE.r' to accommodate SGR 2025 (RH 260323)     + Modified function `plotGMA' to add contours that show the QCS gullies (RH 260324)     + Added new argument 'cohort.label.year' to function `weightBio' for specifying year along x-axis above with cohort labels appear (RH 260326)       - used to label where vertical gaps appear in the bubble plot     + Added more text strings to translate in function `linguaFranca' (RH 260401)
</commit_message>
<xml_diff>
--- a/PBStools/inst/sql/bio.fields.xlsx
+++ b/PBStools/inst/sql/bio.fields.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="120" windowWidth="18195" windowHeight="7740" firstSheet="5" activeTab="20"/>
+    <workbookView xWindow="480" yWindow="120" windowWidth="18195" windowHeight="7740" firstSheet="5" activeTab="15"/>
   </bookViews>
   <sheets>
     <sheet name="bio.fields" sheetId="1" r:id="rId1"/>
@@ -20163,11 +20163,13 @@
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="36">

</xml_diff>